<commit_message>
QR: encode the QR URL column exactly (hyperlink address if linked), no added text
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01GVzT48kTyXj9teBXn6ameE
</commit_message>
<xml_diff>
--- a/sample/sample_guests.xlsx
+++ b/sample/sample_guests.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G15"/>
+  <dimension ref="A1:H15"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -452,6 +452,11 @@
           <t>Room #</t>
         </is>
       </c>
+      <c r="H1" t="inlineStr">
+        <is>
+          <t>QR URL</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="n">
@@ -483,6 +488,11 @@
       <c r="G2" t="n">
         <v>101</v>
       </c>
+      <c r="H2" t="inlineStr">
+        <is>
+          <t>https://example.org/e26/checkin?id=SNR01&amp;name=Sample%20Guest%20One&amp;v=2</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="n">
@@ -514,6 +524,11 @@
       <c r="G3" t="n">
         <v>102</v>
       </c>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t>Open link</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="n">
@@ -545,6 +560,11 @@
       <c r="G4" t="n">
         <v>103</v>
       </c>
+      <c r="H4" t="inlineStr">
+        <is>
+          <t>https://example.org/e26/g/3</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="n">
@@ -576,6 +596,11 @@
       <c r="G5" t="n">
         <v>104</v>
       </c>
+      <c r="H5" t="inlineStr">
+        <is>
+          <t>https://example.org/e26/g/4</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="n">
@@ -607,6 +632,11 @@
       <c r="G6" t="n">
         <v>105</v>
       </c>
+      <c r="H6" t="inlineStr">
+        <is>
+          <t>https://example.org/e26/g/5</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="n">
@@ -638,6 +668,11 @@
       <c r="G7" t="n">
         <v>106</v>
       </c>
+      <c r="H7" t="inlineStr">
+        <is>
+          <t>https://example.org/e26/g/6</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="n">
@@ -669,6 +704,11 @@
       <c r="G8" t="n">
         <v>107</v>
       </c>
+      <c r="H8" t="inlineStr">
+        <is>
+          <t>https://example.org/e26/g/7</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="n">
@@ -700,6 +740,11 @@
       <c r="G9" t="n">
         <v>108</v>
       </c>
+      <c r="H9" t="inlineStr">
+        <is>
+          <t>https://example.org/e26/g/8</t>
+        </is>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="n">
@@ -731,6 +776,11 @@
       <c r="G10" t="n">
         <v>109</v>
       </c>
+      <c r="H10" t="inlineStr">
+        <is>
+          <t>https://example.org/e26/g/9</t>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="A11" t="n">
@@ -762,6 +812,11 @@
       <c r="G11" t="n">
         <v>110</v>
       </c>
+      <c r="H11" t="inlineStr">
+        <is>
+          <t>https://example.org/e26/g/10</t>
+        </is>
+      </c>
     </row>
     <row r="12">
       <c r="A12" t="n">
@@ -793,6 +848,11 @@
       <c r="G12" t="n">
         <v>111</v>
       </c>
+      <c r="H12" t="inlineStr">
+        <is>
+          <t>https://example.org/e26/g/11</t>
+        </is>
+      </c>
     </row>
     <row r="13">
       <c r="A13" t="n">
@@ -824,6 +884,11 @@
       <c r="G13" t="n">
         <v>112</v>
       </c>
+      <c r="H13" t="inlineStr">
+        <is>
+          <t>https://example.org/e26/g/12</t>
+        </is>
+      </c>
     </row>
     <row r="14">
       <c r="A14" t="n">
@@ -855,6 +920,11 @@
       <c r="G14" t="n">
         <v>113</v>
       </c>
+      <c r="H14" t="inlineStr">
+        <is>
+          <t>https://example.org/e26/g/13</t>
+        </is>
+      </c>
     </row>
     <row r="15">
       <c r="A15" t="n">
@@ -886,8 +956,16 @@
       <c r="G15" t="n">
         <v>114</v>
       </c>
+      <c r="H15" t="inlineStr">
+        <is>
+          <t>https://example.org/e26/g/14</t>
+        </is>
+      </c>
     </row>
   </sheetData>
+  <hyperlinks>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H3" r:id="rId1"/>
+  </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
QR: embed the original QR image from the URL unchanged (no regeneration)
- web: fetch via Netlify /qrimg proxy or directly; fallback to picking image files
- python: download + cache, or --qr-images folder
- missing images shown as a dashed box and warned before building

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01GVzT48kTyXj9teBXn6ameE
</commit_message>
<xml_diff>
--- a/sample/sample_guests.xlsx
+++ b/sample/sample_guests.xlsx
@@ -490,7 +490,7 @@
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>https://example.org/e26/checkin?id=SNR01&amp;name=Sample%20Guest%20One&amp;v=2</t>
+          <t>https://example.org/qr/90001_sample.jpeg</t>
         </is>
       </c>
     </row>
@@ -526,7 +526,7 @@
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>Open link</t>
+          <t>https://example.org/qr/90002_sample.jpeg</t>
         </is>
       </c>
     </row>
@@ -562,7 +562,7 @@
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t>https://example.org/e26/g/3</t>
+          <t>https://example.org/qr/90003_sample.jpeg</t>
         </is>
       </c>
     </row>
@@ -598,7 +598,7 @@
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>https://example.org/e26/g/4</t>
+          <t>https://example.org/qr/90004_sample.jpeg</t>
         </is>
       </c>
     </row>
@@ -634,7 +634,7 @@
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>https://example.org/e26/g/5</t>
+          <t>https://example.org/qr/90005_sample.jpeg</t>
         </is>
       </c>
     </row>
@@ -670,7 +670,7 @@
       </c>
       <c r="H7" t="inlineStr">
         <is>
-          <t>https://example.org/e26/g/6</t>
+          <t>https://example.org/qr/90006_sample.jpeg</t>
         </is>
       </c>
     </row>
@@ -706,7 +706,7 @@
       </c>
       <c r="H8" t="inlineStr">
         <is>
-          <t>https://example.org/e26/g/7</t>
+          <t>https://example.org/qr/90007_sample.jpeg</t>
         </is>
       </c>
     </row>
@@ -742,7 +742,7 @@
       </c>
       <c r="H9" t="inlineStr">
         <is>
-          <t>https://example.org/e26/g/8</t>
+          <t>https://example.org/qr/90008_sample.jpeg</t>
         </is>
       </c>
     </row>
@@ -778,7 +778,7 @@
       </c>
       <c r="H10" t="inlineStr">
         <is>
-          <t>https://example.org/e26/g/9</t>
+          <t>https://example.org/qr/90009_sample.jpeg</t>
         </is>
       </c>
     </row>
@@ -814,7 +814,7 @@
       </c>
       <c r="H11" t="inlineStr">
         <is>
-          <t>https://example.org/e26/g/10</t>
+          <t>https://example.org/qr/90010_sample.jpeg</t>
         </is>
       </c>
     </row>
@@ -850,7 +850,7 @@
       </c>
       <c r="H12" t="inlineStr">
         <is>
-          <t>https://example.org/e26/g/11</t>
+          <t>https://example.org/qr/90011_sample.jpeg</t>
         </is>
       </c>
     </row>
@@ -886,7 +886,7 @@
       </c>
       <c r="H13" t="inlineStr">
         <is>
-          <t>https://example.org/e26/g/12</t>
+          <t>https://example.org/qr/90012_sample.jpeg</t>
         </is>
       </c>
     </row>
@@ -922,7 +922,7 @@
       </c>
       <c r="H14" t="inlineStr">
         <is>
-          <t>https://example.org/e26/g/13</t>
+          <t>https://example.org/qr/90013_sample.jpeg</t>
         </is>
       </c>
     </row>
@@ -958,14 +958,11 @@
       </c>
       <c r="H15" t="inlineStr">
         <is>
-          <t>https://example.org/e26/g/14</t>
+          <t>https://example.org/qr/90014_sample.jpeg</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <hyperlinks>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H3" r:id="rId1"/>
-  </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>